<commit_message>
Fixed order issue for hard-tack deeds, added new deeds
</commit_message>
<xml_diff>
--- a/_SourceFiles/DeedInfo-4-The War.xlsx
+++ b/_SourceFiles/DeedInfo-4-The War.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bkckx\Documents\The Lord of the Rings Online\Plugins\CubePlugins\DeedTracker\_SourceFiles\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37192271-8CDC-46BA-AC8E-2A9A36DC3A93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE15603-C866-42EB-B6BA-FE925F2DE886}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28800" yWindow="0" windowWidth="15780" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Common" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="434" uniqueCount="219">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="438" uniqueCount="221">
   <si>
     <t>Save Index</t>
   </si>
@@ -696,6 +696,12 @@
   </si>
   <si>
     <t>Sorceress Slayer -- Tier 4</t>
+  </si>
+  <si>
+    <t>Frame: Season of Renewed Aggression Frame</t>
+  </si>
+  <si>
+    <t>- Season 8: Renewed Aggression -</t>
   </si>
 </sst>
 </file>
@@ -1669,28 +1675,28 @@
           </cell>
         </row>
       </sheetData>
-      <sheetData sheetId="2" refreshError="1"/>
-      <sheetData sheetId="3" refreshError="1"/>
-      <sheetData sheetId="4" refreshError="1"/>
-      <sheetData sheetId="5" refreshError="1"/>
-      <sheetData sheetId="6" refreshError="1"/>
-      <sheetData sheetId="7" refreshError="1"/>
-      <sheetData sheetId="8" refreshError="1"/>
-      <sheetData sheetId="9" refreshError="1"/>
-      <sheetData sheetId="10" refreshError="1"/>
-      <sheetData sheetId="11" refreshError="1"/>
-      <sheetData sheetId="12" refreshError="1"/>
-      <sheetData sheetId="13" refreshError="1"/>
-      <sheetData sheetId="14" refreshError="1"/>
-      <sheetData sheetId="15" refreshError="1"/>
-      <sheetData sheetId="16" refreshError="1"/>
-      <sheetData sheetId="17" refreshError="1"/>
-      <sheetData sheetId="18" refreshError="1"/>
-      <sheetData sheetId="19" refreshError="1"/>
-      <sheetData sheetId="20" refreshError="1"/>
-      <sheetData sheetId="21" refreshError="1"/>
-      <sheetData sheetId="22" refreshError="1"/>
-      <sheetData sheetId="23" refreshError="1"/>
+      <sheetData sheetId="2"/>
+      <sheetData sheetId="3"/>
+      <sheetData sheetId="4"/>
+      <sheetData sheetId="5"/>
+      <sheetData sheetId="6"/>
+      <sheetData sheetId="7"/>
+      <sheetData sheetId="8"/>
+      <sheetData sheetId="9"/>
+      <sheetData sheetId="10"/>
+      <sheetData sheetId="11"/>
+      <sheetData sheetId="12"/>
+      <sheetData sheetId="13"/>
+      <sheetData sheetId="14"/>
+      <sheetData sheetId="15"/>
+      <sheetData sheetId="16"/>
+      <sheetData sheetId="17"/>
+      <sheetData sheetId="18"/>
+      <sheetData sheetId="19"/>
+      <sheetData sheetId="20"/>
+      <sheetData sheetId="21"/>
+      <sheetData sheetId="22"/>
+      <sheetData sheetId="23"/>
     </sheetDataSet>
   </externalBook>
 </externalLink>
@@ -12345,15 +12351,23 @@
       </c>
     </row>
     <row r="23" spans="1:45" x14ac:dyDescent="0.25">
-      <c r="D23" s="2"/>
+      <c r="C23" s="3" t="s">
+        <v>220</v>
+      </c>
+      <c r="D23" s="2" t="s">
+        <v>29</v>
+      </c>
       <c r="N23" s="2"/>
+      <c r="P23">
+        <v>352</v>
+      </c>
       <c r="R23" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [22] = {}; -- </v>
-      </c>
-      <c r="S23" s="1" t="e">
+        <v xml:space="preserve"> [22] = {["CAT_ID"] = 352; }; -- - Season 8: Renewed Aggression -</v>
+      </c>
+      <c r="S23" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>#N/A</v>
+        <v xml:space="preserve"> [22] = {                                         ["TYPE"] = 14; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "- Season 8: Renewed Aggression -"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T23">
         <f t="shared" si="3"/>
@@ -12373,19 +12387,19 @@
       </c>
       <c r="X23" t="str">
         <f t="shared" si="7"/>
-        <v/>
+        <v xml:space="preserve">["CAT_ID"] = 352; </v>
       </c>
       <c r="Y23" s="1" t="str">
         <f t="shared" si="8"/>
         <v xml:space="preserve">                    </v>
       </c>
-      <c r="Z23" t="e">
+      <c r="Z23">
         <f>VLOOKUP(D23,[1]Type!A$2:B$18,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AA23" t="e">
+        <v>14</v>
+      </c>
+      <c r="AA23" t="str">
         <f t="shared" si="9"/>
-        <v>#N/A</v>
+        <v xml:space="preserve">["TYPE"] = 14; </v>
       </c>
       <c r="AB23" t="str">
         <f>IF(NOT(ISBLANK(E23)),VLOOKUP(E23,[1]Type!D$2:E$6,2,FALSE),"")</f>
@@ -12441,7 +12455,7 @@
       </c>
       <c r="AO23" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "- Season 8: Renewed Aggression -"; }; </v>
       </c>
       <c r="AP23" t="str">
         <f t="shared" si="22"/>
@@ -12461,14 +12475,23 @@
       </c>
     </row>
     <row r="24" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>1879531405</v>
+      </c>
+      <c r="C24" t="s">
+        <v>219</v>
+      </c>
+      <c r="D24" t="s">
+        <v>154</v>
+      </c>
       <c r="N24" s="2"/>
       <c r="R24" t="str">
         <f t="shared" si="1"/>
-        <v xml:space="preserve"> [23] = {}; -- </v>
-      </c>
-      <c r="S24" s="1" t="e">
+        <v xml:space="preserve"> [23] = {["ID"] = 1879531405; }; -- Frame: Season of Renewed Aggression Frame</v>
+      </c>
+      <c r="S24" s="1" t="str">
         <f t="shared" si="2"/>
-        <v>#N/A</v>
+        <v xml:space="preserve"> [23] = {["ID"] = 1879531405;                     ["TYPE"] =  7; ["VXP"] = 0; ["LP"] = 0; ["REP"] = 0; ["FACTION"] = 1; ["TIER"] = 0; ["NAME"] = { ["EN"] = "Frame: Season of Renewed Aggression Frame"; }; ["LORE"] = { ["EN"] = ""; }; ["SUMMARY"] = { ["EN"] = ""; }; };</v>
       </c>
       <c r="T24">
         <f t="shared" si="3"/>
@@ -12480,11 +12503,11 @@
       </c>
       <c r="V24" t="str">
         <f t="shared" si="5"/>
-        <v xml:space="preserve">                     </v>
+        <v xml:space="preserve">["ID"] = 1879531405; </v>
       </c>
       <c r="W24" t="str">
         <f t="shared" si="6"/>
-        <v/>
+        <v xml:space="preserve">["ID"] = 1879531405; </v>
       </c>
       <c r="X24" t="str">
         <f t="shared" si="7"/>
@@ -12494,13 +12517,13 @@
         <f t="shared" si="8"/>
         <v xml:space="preserve">                    </v>
       </c>
-      <c r="Z24" t="e">
+      <c r="Z24">
         <f>VLOOKUP(D24,[1]Type!A$2:B$18,2,FALSE)</f>
-        <v>#N/A</v>
-      </c>
-      <c r="AA24" t="e">
+        <v>7</v>
+      </c>
+      <c r="AA24" t="str">
         <f t="shared" si="9"/>
-        <v>#N/A</v>
+        <v xml:space="preserve">["TYPE"] =  7; </v>
       </c>
       <c r="AB24" t="str">
         <f>IF(NOT(ISBLANK(E24)),VLOOKUP(E24,[1]Type!D$2:E$6,2,FALSE),"")</f>
@@ -12556,7 +12579,7 @@
       </c>
       <c r="AO24" t="str">
         <f t="shared" si="21"/>
-        <v xml:space="preserve">["NAME"] = { ["EN"] = ""; }; </v>
+        <v xml:space="preserve">["NAME"] = { ["EN"] = "Frame: Season of Renewed Aggression Frame"; }; </v>
       </c>
       <c r="AP24" t="str">
         <f t="shared" si="22"/>

</xml_diff>